<commit_message>
Update camera code logic in ATS Runner and updated srv files order
</commit_message>
<xml_diff>
--- a/server/ATS/template/green-pcb_template.xlsx
+++ b/server/ATS/template/green-pcb_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ATS\server\ATS\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4843FC22-E5A8-4FC3-8C6D-C8EF15E4F3CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22A5BD96-3A32-44E8-966A-9D9B2A0FAE5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{94096412-2FEB-4621-AAB3-520197C8C40C}"/>
   </bookViews>
@@ -43,9 +43,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Reason</t>
-  </si>
-  <si>
     <t>Remarks</t>
   </si>
   <si>
@@ -62,6 +59,9 @@
   </si>
   <si>
     <t>PREPARED BY:</t>
+  </si>
+  <si>
+    <t>s</t>
   </si>
 </sst>
 </file>
@@ -870,7 +870,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
@@ -926,6 +926,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1289,16 +1292,16 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.5546875" customWidth="1"/>
     <col min="3" max="3" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.21875" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="25" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -1318,7 +1321,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" s="21"/>
       <c r="F3" s="10"/>
@@ -1362,13 +1365,13 @@
         <v>6</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
-      <c r="E8" s="18" t="s">
-        <v>7</v>
+      <c r="E8" s="32" t="s">
+        <v>13</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -1501,12 +1504,12 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="28" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
       <c r="D25" s="30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E25" s="8"/>
       <c r="F25" s="9"/>

</xml_diff>